<commit_message>
Props with Y-sort, held flashlight, editor graphics warnings
- graphics.xlsx Props: sprites placed as map objects (type=prop), drawn from
  the foot tile in the characters' Y-sorted node; solid props collide (walls
  layer, so they also block enemy sight and cutscene path finding), shadow
  casters block light
- LightPresets.shape point / cone; item.xlsx Items.light: a hand-held item
  with a light (dummy flashlight) gives the player a cone that turns with facing
- Map editor: object tool and palette mode with thumbnails, footprint outlines,
  prop inspector, graphics warnings in map settings and red X on unknown tiles;
  shorter graphics tool labels
- Tests: graphics_smoke props/flashlight, map_editor_smoke props/warnings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiles" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LightPresets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DayNight" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LightPresets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DayNight" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -765,7 +766,215 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>prop_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>foot_w</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>foot_h</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>solid</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>casts_shadow</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>tree</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>나무</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>test_tree.png</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>테스트 그림. 줄기 칸만 막고, 잎은 인물 앞을 가림</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>crate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>상자</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>test_crate.png</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>테스트 그림</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>탁자</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>test_table.png</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>테스트 그림 (2칸)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lamp_post</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>가로등</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>test_lamp.png</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>테스트 그림. 빛은 광원을 따로 놓을 것</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -810,6 +1019,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>shape</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -843,6 +1057,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>임시값</t>
         </is>
       </c>
@@ -876,6 +1095,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>임시값</t>
         </is>
       </c>
@@ -909,6 +1133,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>임시값</t>
         </is>
       </c>
@@ -942,6 +1171,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>임시값</t>
         </is>
       </c>
@@ -974,6 +1208,11 @@
         </is>
       </c>
       <c r="G6" t="inlineStr">
+        <is>
+          <t>cone</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>임시값 (지금은 놓인 자리에 고정)</t>
         </is>
@@ -984,7 +1223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1083,7 +1322,6 @@
       <c r="E3" t="n">
         <v>0.1</v>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1135,7 +1373,6 @@
       <c r="E5" t="n">
         <v>0.3</v>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1187,7 +1424,6 @@
       <c r="E7" t="n">
         <v>0.3</v>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1239,7 +1475,6 @@
       <c r="E9" t="n">
         <v>0.15</v>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1330,13 +1565,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1346,7 +1581,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1393,6 +1627,27 @@
       <c r="A9" t="inlineStr">
         <is>
           <t xml:space="preserve">  ambient = 화면 전체에 곱하는 색(어두울수록 어두움), sun_color·sun_energy = 실외 햇빛·달빛 (더해지는 밝기)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Props: 맵 에디터 '오브젝트' 팔레트. file = art/props/ 의 그림(투명 바탕). foot_w·foot_h = 차지하는 칸 (놓은 칸이 왼쪽 아래)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  solid Y = 지나갈 수 없음 + 적 시야도 막음 (벽처럼). casts_shadow Y = 광원 빛을 막음. 앞뒤는 발 위치로 저절로 (인물이 아래에 있으면 앞)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LightPresets.shape: point(둥근 빛) / cone(앞으로 비추는 원뿔 — 손전등). 아이템 item.xlsx Items 의 light 열에 프리셋을 적으면 손에 들 때 플레이어가 그 빛을 들고 다님</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roof tile layer: houses stay covered until the player walks in
New graphics layer 'roof' (Tiles layer=roof, map visual.layers.roof, map
editor palette). Roofs draw above characters and props; each connected
group of roof cells is one house with its own layer, and the house the
player stands under fades out while the others stay covered. Logic
(collision, sight) is unchanged. The map editor shows roofs half
transparent with a 'roof' view filter. Placeholder tiles roof_red and
roof_slate; the city map's buildings get roofs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -752,6 +752,78 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>테스트 타일 (투명 바탕)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>roof_red</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>빨간 지붕</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>roof</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>테스트 타일 — 지붕 층: 인물보다 위, 집 안에 들어가면 그 집 지붕이 사라짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>roof_slate</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>회색 지붕</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>roof</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>테스트 타일 — 지붕 층</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Door and investigate sparkle tiles
Tiles get two non-paint layers: 'door' (closed key, open key_open) and
'marker' (investigate sparkle), plus optional frames/fps for animation.
The shared renderer draws a door sprite on every exit (swapped when the
door opens) and an animated, unshaded sparkle on investigate spots that
disappears once searched; the map editor shows them too and can pick a
door look per exit. Without art the old shapes are drawn. Placeholder
art door_wood, door_wood_open and a 4-frame sparkle.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,16 @@
           <t>note</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>frames</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>fps</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -825,6 +835,120 @@
         <is>
           <t>테스트 타일 — 지붕 층</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>door_wood</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>나무 문</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>door</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>테스트 — 문(exit) 그림, 닫힘. 열린 그림 = 같은 이름 + _open</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>door_wood_open</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>나무 문 (열림)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>door</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>테스트 — door_wood 가 열렸을 때</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sparkle</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>조사 반짝이</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>marker</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>테스트 — 조사 지점(아직 안 한 곳) 표시. atlas_x 부터 오른쪽으로 frames 장, 초당 fps 장. 어두워도 보임</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Map new_america from the village layout plan (300 x 188)
Block-out of the user's village plan: west road (default arrival), north
road, east road toward the church (arrival), south-east road, pond,
houses A-E, shop F, warehouses H and I with roofs (solid; interiors are
separate maps per the plan), fenced yards, fields, trees and street lamps.
Generated by tools/make_new_america.py.

Supporting changes: per-map default floor/wall pictures (visual.default_floor
/ default_wall, map settings in the editor) so big maps stay small; new
placeholder tiles water, fence_wood, forest, roof_brown, roof_green; the
map editor canvas only draws visible cells (big maps stay smooth).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -949,6 +949,186 @@
       </c>
       <c r="J14" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>물</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>wall</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>테스트 — 연못·물 (논리는 벽 # = 못 지나감, 그림자 없음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>fence_wood</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>나무 울타리</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>wall</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>테스트 — 울타리 (논리 벽 #, 빛은 지나감)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>roof_brown</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>갈색 지붕</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>roof</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>테스트 — 창고·부속 건물</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>roof_green</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>초록 지붕</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>roof</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>테스트 — 점포</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>숲</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>wall</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>테스트 — 빽빽한 숲 (논리 벽 #). 맵 기본 벽 그림으로 쓰기 좋음</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Overhead (foreground occlusion) layer: drawn above actors, no collision/sight/light; editor show/hide, overhead-only view, preview opacity, collision overlay; test map
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1342,6 +1342,42 @@
       <c r="H24" t="inlineStr">
         <is>
           <t>커튼을 친 창문</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>overhead_black</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>검은 가림막</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>overhead</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>전경 가림 기본 타일 — 캐릭터 위에 그려지고 충돌·시야·빛 차단 없음</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Overhead follow-up: layer lock, lintel tile, walk-behind furniture rows, seam and NPC order tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1378,6 +1378,42 @@
       <c r="H25" t="inlineStr">
         <is>
           <t>전경 가림 기본 타일 — 캐릭터 위에 그려지고 충돌·시야·빛 차단 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>lintel_wood</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>나무 문틀 상단</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>overhead</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>7</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>문 위 칸에 칠하는 전경 — 문틀 윗부분이 캐릭터 머리 위로 (투명한 위쪽은 벽이 보임)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Curved dirt road tiles: rounded bends and inner corner fills
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1414,6 +1414,294 @@
       <c r="H26" t="inlineStr">
         <is>
           <t>문 위 칸에 칠하는 전경 — 문틀 윗부분이 캐릭터 머리 위로 (투명한 위쪽은 벽이 보임)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>road_curve_ws</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>흙길 굽이 (왼쪽↔아래)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>road_curve_wn</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>흙길 굽이 (왼쪽↔위)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>road_curve_es</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>흙길 굽이 (오른쪽↔아래)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>road_curve_en</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>흙길 굽이 (오른쪽↔위)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>8</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>road_fill_ne</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>흙길 안쪽 모서리 (오른쪽 위)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>9</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>road_fill_nw</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>흙길 안쪽 모서리 (왼쪽 위)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>9</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>road_fill_se</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>흙길 안쪽 모서리 (오른쪽 아래)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>9</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>road_fill_sw</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>흙길 안쪽 모서리 (왼쪽 아래)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>9</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Default P optional everywhere; respawn point R in basecamp for revive/load; camp tent art and MapView above floor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1702,6 +1702,42 @@
       <c r="H34" t="inlineStr">
         <is>
           <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>camp_tent</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>거점 텐트</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>camp</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>10</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>베이스캠프 거점(camp) 그림</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wall lamps: lights can be placed on wall cells with sconce art, lighting the floor in front
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1738,6 +1738,42 @@
       <c r="H35" t="inlineStr">
         <is>
           <t>베이스캠프 거점(camp) 그림</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>wall_lamp</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>벽걸이등</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>lamp</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>10</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>벽에 건 광원(type=light 를 벽 칸에) 그림 — 켜져 있으면 빛 영향 없이 밝게</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2201,6 +2237,44 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>임시값 (지금은 놓인 자리에 고정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>wall_sconce</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>벽걸이등</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#FFC880</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>임시값 — 벽 칸에 놓는 등</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Two-cell-tall doors: Tiles height column, tall door art as the default door
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -500,6 +500,11 @@
           <t>face_rows</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -866,12 +871,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>door_wood</t>
+          <t>door_tall</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>나무 문</t>
+          <t>나무 문 (2칸 높이)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -888,26 +893,29 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>테스트 — 문(exit) 그림, 닫힘. 열린 그림 = 같은 이름 + _open</t>
-        </is>
+          <t>문 그림 16x32 — 문 칸 위 벽 칸까지 올라감 (충돌은 문 칸만)</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>door_wood_open</t>
+          <t>door_tall_open</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>나무 문 (열림)</t>
+          <t>나무 문 (2칸 높이, 열림)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -924,31 +932,34 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>테스트 — door_wood 가 열렸을 때</t>
-        </is>
+          <t>문 그림 16x32 — 문 칸 위 벽 칸까지 올라감 (충돌은 문 칸만)</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sparkle</t>
+          <t>door_wood</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>조사 반짝이</t>
+          <t>나무 문</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>door</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -960,37 +971,31 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>테스트 — 조사 지점(아직 안 한 곳) 표시. atlas_x 부터 오른쪽으로 frames 장, 초당 fps 장. 어두워도 보임</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>4</v>
-      </c>
-      <c r="J14" t="n">
-        <v>6</v>
+          <t>테스트 — 문(exit) 그림, 닫힘. 열린 그림 = 같은 이름 + _open</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>door_wood_open</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>물</t>
+          <t>나무 문 (열림)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>door</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -999,34 +1004,34 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>테스트 — 연못·물 (논리는 벽 # = 못 지나감, 그림자 없음)</t>
+          <t>테스트 — door_wood 가 열렸을 때</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fence_wood</t>
+          <t>sparkle</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>나무 울타리</t>
+          <t>조사 반짝이</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1035,34 +1040,40 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>테스트 — 울타리 (논리 벽 #, 빛은 지나감)</t>
-        </is>
+          <t>테스트 — 조사 지점(아직 안 한 곳) 표시. atlas_x 부터 오른쪽으로 frames 장, 초당 fps 장. 어두워도 보임</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>roof_brown</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>갈색 지붕</t>
+          <t>물</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>roof</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1071,7 +1082,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
         <v>5</v>
@@ -1081,24 +1092,24 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>테스트 — 창고·부속 건물</t>
+          <t>테스트 — 연못·물 (논리는 벽 # = 못 지나감, 그림자 없음)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>roof_green</t>
+          <t>fence_wood</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>초록 지붕</t>
+          <t>나무 울타리</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>roof</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1107,7 +1118,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>5</v>
@@ -1117,24 +1128,24 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>테스트 — 점포</t>
+          <t>테스트 — 울타리 (논리 벽 #, 빛은 지나감)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>forest</t>
+          <t>roof_brown</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>숲</t>
+          <t>갈색 지붕</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>roof</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1143,42 +1154,34 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>테스트 — 빽빽한 숲 (논리 벽 #). 맵 기본 벽 그림으로 쓰기 좋음</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>forest_face</t>
-        </is>
-      </c>
-      <c r="L19" t="n">
-        <v>1</v>
+          <t>테스트 — 창고·부속 건물</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>wall_default_face</t>
+          <t>roof_green</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>돌벽 앞면</t>
+          <t>초록 지붕</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>roof</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1187,29 +1190,29 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>벽 앞면 (비스듬한 탑뷰: 남쪽을 향한 면) — wall_default 의 face</t>
+          <t>테스트 — 점포</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>wall_wood_face</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>나무 벽 앞면</t>
+          <t>숲</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1223,29 +1226,37 @@
         </is>
       </c>
       <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>테스트 — 빽빽한 숲 (논리 벽 #). 맵 기본 벽 그림으로 쓰기 좋음</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>forest_face</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
         <v>1</v>
-      </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>건물 정면 — wall_wood 의 face</t>
-        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>forest_face</t>
+          <t>wall_default_face</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>숲 앞면</t>
+          <t>돌벽 앞면</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1259,34 +1270,34 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>숲 가장자리 앞면 (줄기) — forest 의 face</t>
+          <t>벽 앞면 (비스듬한 탑뷰: 남쪽을 향한 면) — wall_default 의 face</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>window_wood</t>
+          <t>wall_wood_face</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>나무 창문</t>
+          <t>나무 벽 앞면</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>window</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1295,34 +1306,34 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>창문 (맵 물체 type=window). 커튼 친 그림 = window_wood_curtain</t>
+          <t>건물 정면 — wall_wood 의 face</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>window_wood_curtain</t>
+          <t>forest_face</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>나무 창문 (커튼)</t>
+          <t>숲 앞면</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>window</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1331,34 +1342,34 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>커튼을 친 창문</t>
+          <t>숲 가장자리 앞면 (줄기) — forest 의 face</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>overhead_black</t>
+          <t>window_wood</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>검은 가림막</t>
+          <t>나무 창문</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>window</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1367,7 +1378,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
         <v>7</v>
@@ -1377,24 +1388,24 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>전경 가림 기본 타일 — 캐릭터 위에 그려지고 충돌·시야·빛 차단 없음</t>
+          <t>창문 (맵 물체 type=window). 커튼 친 그림 = window_wood_curtain</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lintel_wood</t>
+          <t>window_wood_curtain</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>나무 문틀 상단</t>
+          <t>나무 창문 (커튼)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>window</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1403,7 +1414,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>7</v>
@@ -1413,24 +1424,24 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>문 위 칸에 칠하는 전경 — 문틀 윗부분이 캐릭터 머리 위로 (투명한 위쪽은 벽이 보임)</t>
+          <t>커튼을 친 창문</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>road_curve_ws</t>
+          <t>overhead_black</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>흙길 굽이 (왼쪽↔아래)</t>
+          <t>검은 가림막</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>overhead</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1439,34 +1450,34 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
+          <t>전경 가림 기본 타일 — 캐릭터 위에 그려지고 충돌·시야·빛 차단 없음</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>road_curve_wn</t>
+          <t>lintel_wood</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>흙길 굽이 (왼쪽↔위)</t>
+          <t>나무 문틀 상단</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>overhead</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1475,29 +1486,29 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
+          <t>문 위 칸에 칠하는 전경 — 문틀 윗부분이 캐릭터 머리 위로 (투명한 위쪽은 벽이 보임)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>road_curve_es</t>
+          <t>road_curve_ws</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>흙길 굽이 (오른쪽↔아래)</t>
+          <t>흙길 굽이 (왼쪽↔아래)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1511,7 +1522,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
         <v>8</v>
@@ -1528,12 +1539,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>road_curve_en</t>
+          <t>road_curve_wn</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>흙길 굽이 (오른쪽↔위)</t>
+          <t>흙길 굽이 (왼쪽↔위)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1547,7 +1558,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>8</v>
@@ -1564,12 +1575,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>road_fill_ne</t>
+          <t>road_curve_es</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>흙길 안쪽 모서리 (오른쪽 위)</t>
+          <t>흙길 굽이 (오른쪽↔아래)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1583,29 +1594,29 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>road_fill_nw</t>
+          <t>road_curve_en</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>흙길 안쪽 모서리 (왼쪽 위)</t>
+          <t>흙길 굽이 (오른쪽↔위)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1619,29 +1630,29 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+          <t>곡선 길: 굽는 칸에 (흙이 두 쪽을 잇고 바깥 모서리가 둥근 풀)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>road_fill_se</t>
+          <t>road_fill_ne</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>흙길 안쪽 모서리 (오른쪽 아래)</t>
+          <t>흙길 안쪽 모서리 (오른쪽 위)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1655,7 +1666,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
         <v>9</v>
@@ -1672,12 +1683,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>road_fill_sw</t>
+          <t>road_fill_nw</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>흙길 안쪽 모서리 (왼쪽 아래)</t>
+          <t>흙길 안쪽 모서리 (왼쪽 위)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1691,7 +1702,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>9</v>
@@ -1708,17 +1719,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>camp_tent</t>
+          <t>road_fill_se</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>거점 텐트</t>
+          <t>흙길 안쪽 모서리 (오른쪽 아래)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>camp</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1727,51 +1738,123 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>베이스캠프 거점(camp) 그림</t>
+          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>road_fill_sw</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>흙길 안쪽 모서리 (왼쪽 아래)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>9</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>곡선 길: 굽이 안쪽의 풀 칸에 (모서리를 둥글게 메움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>camp_tent</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>거점 텐트</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>camp</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>10</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>베이스캠프 거점(camp) 그림</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>wall_lamp</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>벽걸이등</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>lamp</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>test_tiles.png</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
         <v>1</v>
       </c>
-      <c r="F36" t="n">
+      <c r="F38" t="n">
         <v>10</v>
       </c>
-      <c r="G36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" t="inlineStr">
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>벽에 건 광원(type=light 를 벽 칸에) 그림 — 켜져 있으면 빛 영향 없이 밝게</t>
         </is>

</xml_diff>

<commit_message>
Back to the 3/4 top-down view; taller wall faces (default 2, wood 3, forest 2 rows)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
House depth shading (hip roofs, wall face edges, ground shadows), stairs tiles and stairs object, make upper/lower floor in map editor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/graphics.xlsx
+++ b/tools/sheets/graphics.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1857,6 +1857,150 @@
       <c r="H38" t="inlineStr">
         <is>
           <t>벽에 건 광원(type=light 를 벽 칸에) 그림 — 켜져 있으면 빛 영향 없이 밝게</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>stairs_stone</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>돌계단</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>11</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>바닥에 칠하는 계단 (지나갈 수 있음, 위가 높은 쪽)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>stairs_wood</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>나무 계단</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>11</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>바닥에 칠하는 계단</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>stairs_up</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>올라가는 계단</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>stairs</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>12</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>계단 물체(층 이동) — 위층으로</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>stairs_down</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>내려가는 계단</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>stairs</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>test_tiles.png</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>12</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>계단 물체(층 이동) — 아래층으로</t>
         </is>
       </c>
     </row>

</xml_diff>